<commit_message>
chore(auto): daily B2B surplus feeds, REST API, compliance, PRs & SEO refresh
</commit_message>
<xml_diff>
--- a/exports/California_Surplus_Feed.xlsx
+++ b/exports/California_Surplus_Feed.xlsx
@@ -588,7 +588,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>2026-08-25 10:41:32</t>
+          <t>2026-08-26 11:20:31</t>
         </is>
       </c>
     </row>
@@ -672,7 +672,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>2026-08-25 10:41:32</t>
+          <t>2026-08-26 11:20:31</t>
         </is>
       </c>
     </row>
@@ -756,7 +756,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>2026-08-25 10:41:32</t>
+          <t>2026-08-26 11:20:31</t>
         </is>
       </c>
     </row>
@@ -840,7 +840,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>2026-08-25 10:41:32</t>
+          <t>2026-08-26 11:20:31</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(auto): daily B2B surplus feeds, REST API, compliance, PRs, SEO & strategy refresh
</commit_message>
<xml_diff>
--- a/exports/California_Surplus_Feed.xlsx
+++ b/exports/California_Surplus_Feed.xlsx
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="O2" t="n">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
@@ -606,7 +606,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>2026-09-06 13:51:06</t>
+          <t>2026-09-07 16:12:10</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
         </is>
       </c>
       <c r="O3" t="n">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
@@ -698,7 +698,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>2026-09-06 13:51:06</t>
+          <t>2026-09-07 16:12:10</t>
         </is>
       </c>
     </row>
@@ -766,7 +766,7 @@
         </is>
       </c>
       <c r="O4" t="n">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="P4" t="inlineStr">
         <is>
@@ -790,7 +790,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>2026-09-06 13:51:06</t>
+          <t>2026-09-07 16:12:10</t>
         </is>
       </c>
     </row>
@@ -858,7 +858,7 @@
         </is>
       </c>
       <c r="O5" t="n">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="P5" t="inlineStr">
         <is>
@@ -882,7 +882,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>2026-09-06 13:51:06</t>
+          <t>2026-09-07 16:12:10</t>
         </is>
       </c>
     </row>

</xml_diff>